<commit_message>
Correct screenshot-derived weekly metrics
</commit_message>
<xml_diff>
--- a/reports/20260720-20260726/城市经理问题闭环填写表_20260720-20260726.xlsx
+++ b/reports/20260720-20260726/城市经理问题闭环填写表_20260720-20260726.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径说明" sheetId="1" r:id="Rc2c78d829ff94cca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部区域" sheetId="2" r:id="R4e6ac68f2a16468e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1区" sheetId="3" r:id="R72403a433ea2432c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2区" sheetId="4" r:id="R5ef16a4297e8417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3区" sheetId="5" r:id="R495b8202929c4864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径说明" sheetId="1" r:id="R8f4fb35bc6c14a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部区域" sheetId="2" r:id="Rbfe00115a2924ce8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1区" sheetId="3" r:id="Recaeb1586c734fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2区" sheetId="4" r:id="R81fb4a25b97c40a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3区" sheetId="5" r:id="Rdc20f93f0fa6476b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -580,125 +580,125 @@
         <x:v>红灯</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
-        <x:v>南阳吾悦</x:v>
+        <x:v>襄阳高新万达</x:v>
       </x:c>
       <x:c r="C2" s="17" t="str">
-        <x:v>完成率53.96%&lt;100%；新签小卡率68.75%&gt;40%</x:v>
+        <x:v>完成率77.70%&lt;100%；新签小卡率66.15%&gt;40%</x:v>
       </x:c>
       <x:c r="D2" s="18" t="str"/>
       <x:c r="E2" s="11" t="str">
+        <x:v>总营收27207；完成率77.70%；新签小/中/大卡43/20/2；新客、老客、续费率待核</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>1. 总营收从26293元变为27207元，增加915元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
+2. 完成率77.70%，距目标还差7809元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
+3. 当前截图已识别新签小卡43张、中卡20张、大卡2张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+      </x:c>
+      <x:c r="G2" s="18" t="str"/>
+    </x:row>
+    <x:row r="3" ht="118" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="str">
+        <x:v>南阳吾悦</x:v>
+      </x:c>
+      <x:c r="C3" s="17" t="str">
+        <x:v>完成率53.96%&lt;100%；新签小卡率68.75%&gt;40%</x:v>
+      </x:c>
+      <x:c r="D3" s="18" t="str"/>
+      <x:c r="E3" s="11" t="str">
         <x:v>总营收19374；完成率53.96%；新签小/中/大卡22/8/2；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F2" s="11" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>1. 总营收从21993元变为19374元，减少2619元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率53.96%，距目标还差16530元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡22张、中卡8张、大卡2张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G2" s="18" t="str"/>
-    </x:row>
-    <x:row r="3" ht="118" customHeight="1">
-      <x:c r="A3" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="str">
+      <x:c r="G3" s="18" t="str"/>
+    </x:row>
+    <x:row r="4" ht="118" customHeight="1">
+      <x:c r="A4" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
         <x:v>许昌魏都万达</x:v>
       </x:c>
-      <x:c r="C3" s="17" t="str">
+      <x:c r="C4" s="17" t="str">
         <x:v>完成率72.05%&lt;100%；新签小卡率57.69%&gt;40%</x:v>
       </x:c>
-      <x:c r="D3" s="18" t="str"/>
-      <x:c r="E3" s="11" t="str">
+      <x:c r="D4" s="18" t="str"/>
+      <x:c r="E4" s="11" t="str">
         <x:v>总营收17482；完成率72.05%；新签小/中/大卡15/11/0；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F3" s="11" t="str">
+      <x:c r="F4" s="11" t="str">
         <x:v>1. 本周总营收17482元，请列出贡献最大的3笔订单、员工和卡型。
 2. 完成率72.05%，距目标还差6782元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡15张、中卡11张、大卡0张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str"/>
-    </x:row>
-    <x:row r="4" ht="118" customHeight="1">
-      <x:c r="A4" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B4" s="11" t="str">
+      <x:c r="G4" s="18" t="str"/>
+    </x:row>
+    <x:row r="5" ht="118" customHeight="1">
+      <x:c r="A5" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
         <x:v>商丘万达</x:v>
       </x:c>
-      <x:c r="C4" s="17" t="str">
+      <x:c r="C5" s="17" t="str">
         <x:v>完成率82.39%&lt;100%；新签小卡率58.33%&gt;40%</x:v>
       </x:c>
-      <x:c r="D4" s="18" t="str"/>
-      <x:c r="E4" s="11" t="str">
+      <x:c r="D5" s="18" t="str"/>
+      <x:c r="E5" s="11" t="str">
         <x:v>总营收17406；完成率82.39%；新签小/中/大卡14/5/5；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F4" s="11" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>1. 总营收从15461元变为17406元，增加1945元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率82.39%，距目标还差3720元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡14张、中卡5张、大卡5张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G4" s="18" t="str"/>
-    </x:row>
-    <x:row r="5" ht="118" customHeight="1">
-      <x:c r="A5" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B5" s="11" t="str">
+      <x:c r="G5" s="18" t="str"/>
+    </x:row>
+    <x:row r="6" ht="118" customHeight="1">
+      <x:c r="A6" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
         <x:v>南阳万达</x:v>
       </x:c>
-      <x:c r="C5" s="17" t="str">
-        <x:v>完成率49.01%&lt;100%；新签小卡率65.22%&gt;40%</x:v>
-      </x:c>
-      <x:c r="D5" s="18" t="str"/>
-      <x:c r="E5" s="11" t="str">
-        <x:v>总营收14716；完成率49.01%；新签小/中/大卡15/5/3；新客、老客、续费率待核</x:v>
-      </x:c>
-      <x:c r="F5" s="11" t="str">
+      <x:c r="C6" s="17" t="str">
+        <x:v>完成率49.01%&lt;100%；新签小卡率66.67%&gt;40%</x:v>
+      </x:c>
+      <x:c r="D6" s="18" t="str"/>
+      <x:c r="E6" s="11" t="str">
+        <x:v>总营收14716；完成率49.01%；新签小/中/大卡18/6/3；新客、老客、续费率待核</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
         <x:v>1. 总营收从24886元变为14716元，减少10170元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率49.01%，距目标还差15311元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡15张、中卡5张、大卡3张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
-      </x:c>
-      <x:c r="G5" s="18" t="str"/>
-    </x:row>
-    <x:row r="6" ht="118" customHeight="1">
-      <x:c r="A6" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="str">
+3. 当前截图已识别新签小卡18张、中卡6张、大卡3张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+      </x:c>
+      <x:c r="G6" s="18" t="str"/>
+    </x:row>
+    <x:row r="7" ht="118" customHeight="1">
+      <x:c r="A7" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
         <x:v>信阳万达</x:v>
       </x:c>
-      <x:c r="C6" s="17" t="str">
+      <x:c r="C7" s="17" t="str">
         <x:v>完成率66.01%&lt;100%；新签小卡率60.71%&gt;40%</x:v>
       </x:c>
-      <x:c r="D6" s="18" t="str"/>
-      <x:c r="E6" s="11" t="str">
+      <x:c r="D7" s="18" t="str"/>
+      <x:c r="E7" s="11" t="str">
         <x:v>总营收11921；完成率66.01%；新签小/中/大卡17/10/1；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F6" s="11" t="str">
+      <x:c r="F7" s="11" t="str">
         <x:v>1. 总营收从10690元变为11921元，增加1231元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率66.01%，距目标还差6139元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡17张、中卡10张、大卡1张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G6" s="18" t="str"/>
-    </x:row>
-    <x:row r="7" ht="118" customHeight="1">
-      <x:c r="A7" s="22" t="str">
-        <x:v>黄灯</x:v>
-      </x:c>
-      <x:c r="B7" s="11" t="str">
-        <x:v>襄阳高新万达</x:v>
-      </x:c>
-      <x:c r="C7" s="17" t="str">
-        <x:v>完成率77.70%&lt;100%；新签小卡率53.13%&gt;40%</x:v>
-      </x:c>
-      <x:c r="D7" s="18" t="str"/>
-      <x:c r="E7" s="11" t="str">
-        <x:v>总营收27207；完成率77.70%；新签小/中/大卡34/28/2；新客、老客、续费率待核</x:v>
-      </x:c>
-      <x:c r="F7" s="11" t="str">
-        <x:v>1. 总营收从26293元变为27207元，增加915元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
-2. 完成率77.70%，距目标还差7809元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡34张、中卡28张、大卡2张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
-      </x:c>
       <x:c r="G7" s="18" t="str"/>
     </x:row>
     <x:row r="8" ht="118" customHeight="1">
@@ -706,104 +706,104 @@
         <x:v>红灯</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
-        <x:v>洛阳中州万达</x:v>
+        <x:v>洛阳泉舜</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
-        <x:v>完成率76.64%&lt;100%；新签小卡率74.47%&gt;40%</x:v>
+        <x:v>完成率77.40%&lt;100%；新签小卡率56.41%&gt;40%</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str"/>
       <x:c r="E8" s="11" t="str">
+        <x:v>总营收34016；完成率77.40%；新签小/中/大卡22/11/6；新客、老客、续费率待核</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>1. 总营收从65202元变为34016元，减少31186元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
+2. 完成率77.40%，距目标还差9934元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
+3. 当前截图已识别新签小卡22张、中卡11张、大卡6张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+      </x:c>
+      <x:c r="G8" s="18" t="str"/>
+    </x:row>
+    <x:row r="9" ht="118" customHeight="1">
+      <x:c r="A9" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>洛阳中州万达</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>完成率76.64%&lt;100%；新签小卡率74.47%&gt;40%</x:v>
+      </x:c>
+      <x:c r="D9" s="18" t="str"/>
+      <x:c r="E9" s="11" t="str">
         <x:v>总营收18990；完成率76.64%；新签小/中/大卡35/12/0；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F8" s="11" t="str">
+      <x:c r="F9" s="11" t="str">
         <x:v>1. 总营收从15679元变为18990元，增加3311元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率76.64%，距目标还差5788元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡35张、中卡12张、大卡0张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G8" s="18" t="str"/>
-    </x:row>
-    <x:row r="9" ht="118" customHeight="1">
-      <x:c r="A9" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B9" s="11" t="str">
+      <x:c r="G9" s="18" t="str"/>
+    </x:row>
+    <x:row r="10" ht="118" customHeight="1">
+      <x:c r="A10" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
         <x:v>郑州惠济万达</x:v>
       </x:c>
-      <x:c r="C9" s="17" t="str">
+      <x:c r="C10" s="17" t="str">
         <x:v>完成率56.45%&lt;100%</x:v>
       </x:c>
-      <x:c r="D9" s="18" t="str"/>
-      <x:c r="E9" s="11" t="str">
+      <x:c r="D10" s="18" t="str"/>
+      <x:c r="E10" s="11" t="str">
         <x:v>总营收12223；完成率56.45%；新签小/中/大卡4/11/1；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F9" s="11" t="str">
+      <x:c r="F10" s="11" t="str">
         <x:v>1. 总营收从17422元变为12223元，减少5199元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率56.45%，距目标还差9431元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡4张、中卡11张、大卡1张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G9" s="18" t="str"/>
-    </x:row>
-    <x:row r="10" ht="118" customHeight="1">
-      <x:c r="A10" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B10" s="11" t="str">
+      <x:c r="G10" s="18" t="str"/>
+    </x:row>
+    <x:row r="11" ht="118" customHeight="1">
+      <x:c r="A11" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
         <x:v>新乡万达</x:v>
       </x:c>
-      <x:c r="C10" s="17" t="str">
+      <x:c r="C11" s="17" t="str">
         <x:v>完成率61.88%&lt;100%；新签小卡率42.86%&gt;40%</x:v>
       </x:c>
-      <x:c r="D10" s="18" t="str"/>
-      <x:c r="E10" s="11" t="str">
+      <x:c r="D11" s="18" t="str"/>
+      <x:c r="E11" s="11" t="str">
         <x:v>总营收11731；完成率61.88%；新签小/中/大卡3/4/0；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F10" s="11" t="str">
+      <x:c r="F11" s="11" t="str">
         <x:v>1. 总营收从14444元变为11731元，减少2713元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率61.88%，距目标还差7228元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡3张、中卡4张、大卡0张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G10" s="18" t="str"/>
-    </x:row>
-    <x:row r="11" ht="118" customHeight="1">
-      <x:c r="A11" s="22" t="str">
+      <x:c r="G11" s="18" t="str"/>
+    </x:row>
+    <x:row r="12" ht="118" customHeight="1">
+      <x:c r="A12" s="22" t="str">
         <x:v>黄灯</x:v>
       </x:c>
-      <x:c r="B11" s="11" t="str">
+      <x:c r="B12" s="11" t="str">
         <x:v>焦作万达</x:v>
       </x:c>
-      <x:c r="C11" s="17" t="str">
+      <x:c r="C12" s="17" t="str">
         <x:v>完成率91.25%&lt;100%；新签小卡率54.76%&gt;40%</x:v>
       </x:c>
-      <x:c r="D11" s="18" t="str"/>
-      <x:c r="E11" s="11" t="str">
+      <x:c r="D12" s="18" t="str"/>
+      <x:c r="E12" s="11" t="str">
         <x:v>总营收36882；完成率91.25%；新签小/中/大卡23/19/0；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F11" s="11" t="str">
+      <x:c r="F12" s="11" t="str">
         <x:v>1. 总营收从32869元变为36882元，增加4014元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率91.25%，距目标还差3537元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡23张、中卡19张、大卡0张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G11" s="18" t="str"/>
-    </x:row>
-    <x:row r="12" ht="118" customHeight="1">
-      <x:c r="A12" s="22" t="str">
-        <x:v>黄灯</x:v>
-      </x:c>
-      <x:c r="B12" s="11" t="str">
-        <x:v>洛阳泉舜</x:v>
-      </x:c>
-      <x:c r="C12" s="17" t="str">
-        <x:v>完成率77.40%&lt;100%；新签小卡率53.49%&gt;40%</x:v>
-      </x:c>
-      <x:c r="D12" s="18" t="str"/>
-      <x:c r="E12" s="11" t="str">
-        <x:v>总营收34016；完成率77.40%；新签小/中/大卡23/14/6；新客、老客、续费率待核</x:v>
-      </x:c>
-      <x:c r="F12" s="11" t="str">
-        <x:v>1. 总营收从65202元变为34016元，减少31186元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
-2. 完成率77.40%，距目标还差9934元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡23张、中卡14张、大卡6张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
-      </x:c>
       <x:c r="G12" s="18" t="str"/>
     </x:row>
     <x:row r="13" ht="118" customHeight="1">
@@ -818,12 +818,12 @@
       </x:c>
       <x:c r="D13" s="18" t="str"/>
       <x:c r="E13" s="11" t="str">
-        <x:v>总营收16093；完成率84.85%；新签小/中/大卡1/9/12；新客、老客、续费率待核</x:v>
+        <x:v>总营收16093；完成率84.85%；新签小/中/大卡1/10/16；新客、老客、续费率待核</x:v>
       </x:c>
       <x:c r="F13" s="11" t="str">
         <x:v>1. 总营收从13881元变为16093元，增加2212元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率84.85%，距目标还差2873元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡1张、中卡9张、大卡12张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+3. 当前截图已识别新签小卡1张、中卡10张、大卡16张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str"/>
     </x:row>
@@ -839,12 +839,12 @@
       </x:c>
       <x:c r="D14" s="18" t="str"/>
       <x:c r="E14" s="11" t="str">
-        <x:v>总营收27184；完成率133.32%；新签小/中/大卡9/21/4；新客、老客、续费率待核</x:v>
+        <x:v>总营收27184；完成率133.32%；新签小/中/大卡9/21/5；新客、老客、续费率待核</x:v>
       </x:c>
       <x:c r="F14" s="11" t="str">
         <x:v>1. 总营收从14630元变为27184元，增加12553元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率133.32%，距目标还差0元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡9张、中卡21张、大卡4张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+3. 当前截图已识别新签小卡9张、中卡21张、大卡5张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str"/>
     </x:row>
@@ -977,7 +977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reafdab75c8d04657"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R967cddafbe644f1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1023,131 +1023,131 @@
         <x:v>红灯</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
-        <x:v>南阳吾悦</x:v>
+        <x:v>襄阳高新万达</x:v>
       </x:c>
       <x:c r="C2" s="17" t="str">
-        <x:v>完成率53.96%&lt;100%；新签小卡率68.75%&gt;40%</x:v>
+        <x:v>完成率77.70%&lt;100%；新签小卡率66.15%&gt;40%</x:v>
       </x:c>
       <x:c r="D2" s="18" t="str"/>
       <x:c r="E2" s="11" t="str">
+        <x:v>总营收27207；完成率77.70%；新签小/中/大卡43/20/2；新客、老客、续费率待核</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>1. 总营收从26293元变为27207元，增加915元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
+2. 完成率77.70%，距目标还差7809元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
+3. 当前截图已识别新签小卡43张、中卡20张、大卡2张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+      </x:c>
+      <x:c r="G2" s="18" t="str"/>
+    </x:row>
+    <x:row r="3" ht="118" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="str">
+        <x:v>南阳吾悦</x:v>
+      </x:c>
+      <x:c r="C3" s="17" t="str">
+        <x:v>完成率53.96%&lt;100%；新签小卡率68.75%&gt;40%</x:v>
+      </x:c>
+      <x:c r="D3" s="18" t="str"/>
+      <x:c r="E3" s="11" t="str">
         <x:v>总营收19374；完成率53.96%；新签小/中/大卡22/8/2；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F2" s="11" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>1. 总营收从21993元变为19374元，减少2619元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率53.96%，距目标还差16530元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡22张、中卡8张、大卡2张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G2" s="18" t="str"/>
-    </x:row>
-    <x:row r="3" ht="118" customHeight="1">
-      <x:c r="A3" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="str">
+      <x:c r="G3" s="18" t="str"/>
+    </x:row>
+    <x:row r="4" ht="118" customHeight="1">
+      <x:c r="A4" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
         <x:v>许昌魏都万达</x:v>
       </x:c>
-      <x:c r="C3" s="17" t="str">
+      <x:c r="C4" s="17" t="str">
         <x:v>完成率72.05%&lt;100%；新签小卡率57.69%&gt;40%</x:v>
       </x:c>
-      <x:c r="D3" s="18" t="str"/>
-      <x:c r="E3" s="11" t="str">
+      <x:c r="D4" s="18" t="str"/>
+      <x:c r="E4" s="11" t="str">
         <x:v>总营收17482；完成率72.05%；新签小/中/大卡15/11/0；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F3" s="11" t="str">
+      <x:c r="F4" s="11" t="str">
         <x:v>1. 本周总营收17482元，请列出贡献最大的3笔订单、员工和卡型。
 2. 完成率72.05%，距目标还差6782元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡15张、中卡11张、大卡0张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str"/>
-    </x:row>
-    <x:row r="4" ht="118" customHeight="1">
-      <x:c r="A4" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B4" s="11" t="str">
+      <x:c r="G4" s="18" t="str"/>
+    </x:row>
+    <x:row r="5" ht="118" customHeight="1">
+      <x:c r="A5" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
         <x:v>商丘万达</x:v>
       </x:c>
-      <x:c r="C4" s="17" t="str">
+      <x:c r="C5" s="17" t="str">
         <x:v>完成率82.39%&lt;100%；新签小卡率58.33%&gt;40%</x:v>
       </x:c>
-      <x:c r="D4" s="18" t="str"/>
-      <x:c r="E4" s="11" t="str">
+      <x:c r="D5" s="18" t="str"/>
+      <x:c r="E5" s="11" t="str">
         <x:v>总营收17406；完成率82.39%；新签小/中/大卡14/5/5；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F4" s="11" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>1. 总营收从15461元变为17406元，增加1945元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率82.39%，距目标还差3720元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡14张、中卡5张、大卡5张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G4" s="18" t="str"/>
-    </x:row>
-    <x:row r="5" ht="118" customHeight="1">
-      <x:c r="A5" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B5" s="11" t="str">
+      <x:c r="G5" s="18" t="str"/>
+    </x:row>
+    <x:row r="6" ht="118" customHeight="1">
+      <x:c r="A6" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
         <x:v>南阳万达</x:v>
       </x:c>
-      <x:c r="C5" s="17" t="str">
-        <x:v>完成率49.01%&lt;100%；新签小卡率65.22%&gt;40%</x:v>
-      </x:c>
-      <x:c r="D5" s="18" t="str"/>
-      <x:c r="E5" s="11" t="str">
-        <x:v>总营收14716；完成率49.01%；新签小/中/大卡15/5/3；新客、老客、续费率待核</x:v>
-      </x:c>
-      <x:c r="F5" s="11" t="str">
+      <x:c r="C6" s="17" t="str">
+        <x:v>完成率49.01%&lt;100%；新签小卡率66.67%&gt;40%</x:v>
+      </x:c>
+      <x:c r="D6" s="18" t="str"/>
+      <x:c r="E6" s="11" t="str">
+        <x:v>总营收14716；完成率49.01%；新签小/中/大卡18/6/3；新客、老客、续费率待核</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
         <x:v>1. 总营收从24886元变为14716元，减少10170元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率49.01%，距目标还差15311元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡15张、中卡5张、大卡3张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
-      </x:c>
-      <x:c r="G5" s="18" t="str"/>
-    </x:row>
-    <x:row r="6" ht="118" customHeight="1">
-      <x:c r="A6" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="str">
+3. 当前截图已识别新签小卡18张、中卡6张、大卡3张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+      </x:c>
+      <x:c r="G6" s="18" t="str"/>
+    </x:row>
+    <x:row r="7" ht="118" customHeight="1">
+      <x:c r="A7" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
         <x:v>信阳万达</x:v>
       </x:c>
-      <x:c r="C6" s="17" t="str">
+      <x:c r="C7" s="17" t="str">
         <x:v>完成率66.01%&lt;100%；新签小卡率60.71%&gt;40%</x:v>
       </x:c>
-      <x:c r="D6" s="18" t="str"/>
-      <x:c r="E6" s="11" t="str">
+      <x:c r="D7" s="18" t="str"/>
+      <x:c r="E7" s="11" t="str">
         <x:v>总营收11921；完成率66.01%；新签小/中/大卡17/10/1；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F6" s="11" t="str">
+      <x:c r="F7" s="11" t="str">
         <x:v>1. 总营收从10690元变为11921元，增加1231元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率66.01%，距目标还差6139元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡17张、中卡10张、大卡1张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G6" s="18" t="str"/>
-    </x:row>
-    <x:row r="7" ht="118" customHeight="1">
-      <x:c r="A7" s="22" t="str">
-        <x:v>黄灯</x:v>
-      </x:c>
-      <x:c r="B7" s="11" t="str">
-        <x:v>襄阳高新万达</x:v>
-      </x:c>
-      <x:c r="C7" s="17" t="str">
-        <x:v>完成率77.70%&lt;100%；新签小卡率53.13%&gt;40%</x:v>
-      </x:c>
-      <x:c r="D7" s="18" t="str"/>
-      <x:c r="E7" s="11" t="str">
-        <x:v>总营收27207；完成率77.70%；新签小/中/大卡34/28/2；新客、老客、续费率待核</x:v>
-      </x:c>
-      <x:c r="F7" s="11" t="str">
-        <x:v>1. 总营收从26293元变为27207元，增加915元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
-2. 完成率77.70%，距目标还差7809元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡34张、中卡28张、大卡2张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
-      </x:c>
       <x:c r="G7" s="18" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98433bbf5c6f41f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1f8cffc788940cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1193,104 +1193,104 @@
         <x:v>红灯</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
-        <x:v>洛阳中州万达</x:v>
+        <x:v>洛阳泉舜</x:v>
       </x:c>
       <x:c r="C2" s="17" t="str">
-        <x:v>完成率76.64%&lt;100%；新签小卡率74.47%&gt;40%</x:v>
+        <x:v>完成率77.40%&lt;100%；新签小卡率56.41%&gt;40%</x:v>
       </x:c>
       <x:c r="D2" s="18" t="str"/>
       <x:c r="E2" s="11" t="str">
+        <x:v>总营收34016；完成率77.40%；新签小/中/大卡22/11/6；新客、老客、续费率待核</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>1. 总营收从65202元变为34016元，减少31186元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
+2. 完成率77.40%，距目标还差9934元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
+3. 当前截图已识别新签小卡22张、中卡11张、大卡6张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+      </x:c>
+      <x:c r="G2" s="18" t="str"/>
+    </x:row>
+    <x:row r="3" ht="118" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="str">
+        <x:v>洛阳中州万达</x:v>
+      </x:c>
+      <x:c r="C3" s="17" t="str">
+        <x:v>完成率76.64%&lt;100%；新签小卡率74.47%&gt;40%</x:v>
+      </x:c>
+      <x:c r="D3" s="18" t="str"/>
+      <x:c r="E3" s="11" t="str">
         <x:v>总营收18990；完成率76.64%；新签小/中/大卡35/12/0；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F2" s="11" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>1. 总营收从15679元变为18990元，增加3311元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率76.64%，距目标还差5788元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡35张、中卡12张、大卡0张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G2" s="18" t="str"/>
-    </x:row>
-    <x:row r="3" ht="118" customHeight="1">
-      <x:c r="A3" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="str">
+      <x:c r="G3" s="18" t="str"/>
+    </x:row>
+    <x:row r="4" ht="118" customHeight="1">
+      <x:c r="A4" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
         <x:v>郑州惠济万达</x:v>
       </x:c>
-      <x:c r="C3" s="17" t="str">
+      <x:c r="C4" s="17" t="str">
         <x:v>完成率56.45%&lt;100%</x:v>
       </x:c>
-      <x:c r="D3" s="18" t="str"/>
-      <x:c r="E3" s="11" t="str">
+      <x:c r="D4" s="18" t="str"/>
+      <x:c r="E4" s="11" t="str">
         <x:v>总营收12223；完成率56.45%；新签小/中/大卡4/11/1；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F3" s="11" t="str">
+      <x:c r="F4" s="11" t="str">
         <x:v>1. 总营收从17422元变为12223元，减少5199元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率56.45%，距目标还差9431元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡4张、中卡11张、大卡1张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G3" s="18" t="str"/>
-    </x:row>
-    <x:row r="4" ht="118" customHeight="1">
-      <x:c r="A4" s="16" t="str">
-        <x:v>红灯</x:v>
-      </x:c>
-      <x:c r="B4" s="11" t="str">
+      <x:c r="G4" s="18" t="str"/>
+    </x:row>
+    <x:row r="5" ht="118" customHeight="1">
+      <x:c r="A5" s="16" t="str">
+        <x:v>红灯</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
         <x:v>新乡万达</x:v>
       </x:c>
-      <x:c r="C4" s="17" t="str">
+      <x:c r="C5" s="17" t="str">
         <x:v>完成率61.88%&lt;100%；新签小卡率42.86%&gt;40%</x:v>
       </x:c>
-      <x:c r="D4" s="18" t="str"/>
-      <x:c r="E4" s="11" t="str">
+      <x:c r="D5" s="18" t="str"/>
+      <x:c r="E5" s="11" t="str">
         <x:v>总营收11731；完成率61.88%；新签小/中/大卡3/4/0；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F4" s="11" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>1. 总营收从14444元变为11731元，减少2713元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率61.88%，距目标还差7228元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡3张、中卡4张、大卡0张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G4" s="18" t="str"/>
-    </x:row>
-    <x:row r="5" ht="118" customHeight="1">
-      <x:c r="A5" s="22" t="str">
+      <x:c r="G5" s="18" t="str"/>
+    </x:row>
+    <x:row r="6" ht="118" customHeight="1">
+      <x:c r="A6" s="22" t="str">
         <x:v>黄灯</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>焦作万达</x:v>
       </x:c>
-      <x:c r="C5" s="17" t="str">
+      <x:c r="C6" s="17" t="str">
         <x:v>完成率91.25%&lt;100%；新签小卡率54.76%&gt;40%</x:v>
       </x:c>
-      <x:c r="D5" s="18" t="str"/>
-      <x:c r="E5" s="11" t="str">
+      <x:c r="D6" s="18" t="str"/>
+      <x:c r="E6" s="11" t="str">
         <x:v>总营收36882；完成率91.25%；新签小/中/大卡23/19/0；新客、老客、续费率待核</x:v>
       </x:c>
-      <x:c r="F5" s="11" t="str">
+      <x:c r="F6" s="11" t="str">
         <x:v>1. 总营收从32869元变为36882元，增加4014元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率91.25%，距目标还差3537元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
 3. 当前截图已识别新签小卡23张、中卡19张、大卡0张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
-      <x:c r="G5" s="18" t="str"/>
-    </x:row>
-    <x:row r="6" ht="118" customHeight="1">
-      <x:c r="A6" s="22" t="str">
-        <x:v>黄灯</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="str">
-        <x:v>洛阳泉舜</x:v>
-      </x:c>
-      <x:c r="C6" s="17" t="str">
-        <x:v>完成率77.40%&lt;100%；新签小卡率53.49%&gt;40%</x:v>
-      </x:c>
-      <x:c r="D6" s="18" t="str"/>
-      <x:c r="E6" s="11" t="str">
-        <x:v>总营收34016；完成率77.40%；新签小/中/大卡23/14/6；新客、老客、续费率待核</x:v>
-      </x:c>
-      <x:c r="F6" s="11" t="str">
-        <x:v>1. 总营收从65202元变为34016元，减少31186元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
-2. 完成率77.40%，距目标还差9934元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡23张、中卡14张、大卡6张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
-      </x:c>
       <x:c r="G6" s="18" t="str"/>
     </x:row>
     <x:row r="7" ht="118" customHeight="1">
@@ -1305,12 +1305,12 @@
       </x:c>
       <x:c r="D7" s="18" t="str"/>
       <x:c r="E7" s="11" t="str">
-        <x:v>总营收16093；完成率84.85%；新签小/中/大卡1/9/12；新客、老客、续费率待核</x:v>
+        <x:v>总营收16093；完成率84.85%；新签小/中/大卡1/10/16；新客、老客、续费率待核</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
         <x:v>1. 总营收从13881元变为16093元，增加2212元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率84.85%，距目标还差2873元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡1张、中卡9张、大卡12张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+3. 当前截图已识别新签小卡1张、中卡10张、大卡16张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
       <x:c r="G7" s="18" t="str"/>
     </x:row>
@@ -1326,19 +1326,19 @@
       </x:c>
       <x:c r="D8" s="18" t="str"/>
       <x:c r="E8" s="11" t="str">
-        <x:v>总营收27184；完成率133.32%；新签小/中/大卡9/21/4；新客、老客、续费率待核</x:v>
+        <x:v>总营收27184；完成率133.32%；新签小/中/大卡9/21/5；新客、老客、续费率待核</x:v>
       </x:c>
       <x:c r="F8" s="11" t="str">
         <x:v>1. 总营收从14630元变为27184元，增加12553元。请拆出影响最大的3笔订单、员工和卡型；剔除这3笔后真实趋势是什么？
 2. 完成率133.32%，距目标还差0元。下周准备用新客量、客单价还是续卡拉齐？请给责任人、每日动作量和预计补回金额。
-3. 当前截图已识别新签小卡9张、中卡21张、大卡4张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
+3. 当前截图已识别新签小卡9张、中卡21张、大卡5张。请抽查最近5笔小卡成交：客户为什么没升卡、谁接待、卡在哪句话或报价顺序？</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f0ae8b533704841"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fe98c04eed94a36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1508,7 +1508,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9af509bcc594590"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d69b70434bd454e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>